<commit_message>
update baru 16 juli
</commit_message>
<xml_diff>
--- a/output/CMO_LK-000019_202607.xlsx
+++ b/output/CMO_LK-000019_202607.xlsx
@@ -7,7 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="CMO" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Stock" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Outsell" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Avg Outsell" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3736,4 +3738,4806 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C144"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Kode SKU JIM</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Nama SKU JIM</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Qty Karton</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>AGA080391</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>AGANOL LAVENDER  /1L</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>AGA080991</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>AGANOL LAVENDER  /630ML</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>AGA101391A</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>AGANOL FLORAL  /1L</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>AGA101392</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>AGANOL LEMON FRESH  /1L</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>AGA101393</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>AGANOL MORNING FRESH W/ LEMONGRASS  /1L</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>AGA101593</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>AGANOL MORNING FRESH W/ LEMONGRASS  /3,7LT</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>AGA101991B</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>AGANOL FLORAL  /630ML</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>AGA101992</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>AGANOL LEMON  /630ML</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>BBS106390</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>BABY SOFT   /1L</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>BBS106590</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>BABY SOFT   /3,7LT</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>BCL100390</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>YURI BATHROOM CLEANER   /375ML</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>BIO112290</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>BIOSOFT   /375ML</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>BIO113921</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>BIOSOFT HIJAB DETERGENT+SOFTENER OCEAN FRESH /630ML</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>BLE123390</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>YURI BLEACH MORNING FRESH  /1L</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>BLE123392</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>YURI BLEACH LEMON  /1L</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>BLE123590</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>YURI BLEACH MORNING FRESH  /3,7LT</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>BLE123592</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>YURI BLEACH LEMON  /3,7LT</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>DBD750291</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>BABYDEE BODYWASH &amp; SHAMPOO MILK /200ML</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>DBD750292</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>BABYDEE BODYWASH &amp; SHAMPOO HONEY /200ML</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>DBD750931</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>BABY DEE BODYWASH &amp; SHAMPOO NATURAL MILK &amp; LAVENDER EXTRACT FOAMING 600ML</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>DBD750932</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>BABY DEE BODYWASH &amp; SHAMPOO NATURAL HONEY&amp;CHAMOMILE EXTRACT FOAMING 600ML</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>DBD761261</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>BABYDEE TRAVEL PACK MILK</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>DBD761262</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>BABYDEE TRAVEL PACK HONEY</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>DBD761291</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>BABYDEE TALCUM MILK /200GR</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>DBD794092</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>BABYDEE BABY LOTION HONEY /50ML</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>DBD794191</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>BABYDEE BABY LOTION MILK /100ML</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>DBW640291</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>DEEDEE BODYWASH APPLE /225ML</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>DBW640292</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>DEEDEE BODYWASH GRAPE /225ML</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>DBW640293</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>DEEDEE BODYWASH ORANGE /225ML</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>DBW640294</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>DEEDEE BODYWASH STRAWBERRY /225ML</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>DBW640991</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>DEEDEE BODYWASH APPLE /200ML</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>DBW640992</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>DEEDEE BODYWASH GRAPE /200ML</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>DBW640993</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>DEEDEE BODYWASH ORANGE /200ML</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>DBW640994</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>DEEDEE BODYWASH STRAWBERRY /200ML</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>DDM497193</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>DEEDEE LOT. PENOLAK NYAMUK ORANGE /50GR</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>DDM497195</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>DEEDEE LOT. PENOLAK NYAMUK GUAVA /50GR</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>DDP356281A</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>DEE DEE SHAMPOO (P) - APPLE BTL/250ML (POKEMON)</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>DDP356282A</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>DEE DEE SHAMPOO (P) - GRAPE BTL/250ML (POKEMON)</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>DDP356283A</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>DEE DEE SHAMPOO (P) - ORANGE BTL/250ML (POKEMON)</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>DDP356284A</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>DEE DEE SHAMPOO (P) - STRAWBERRY BTL/250ML (POKEMON)</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>DDR356191A</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>DEEDEE SHAMPOO APPLE /45ML</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>DDR356192A</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>DEEDEE SHAMPOO GRAPE /45ML</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>DDR356193A</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>DEEDEE SHAMPOO ORANGE /45ML</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>DDR356194A</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>DEEDEE SHAMPOO STRAWBERRY /45ML</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>DDR356291A</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>DEE DEE SHAMPOO (RF) - APPLE BTL/250ML (POKEMON)</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>DDR356292A</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>DEE DEE SHAMPOO (RF) - GRAPE BTL/250ML (POKEMON)</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>DDR356293A</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>DEE DEE SHAMPOO (RF) - ORANGE BTL/250ML (POKEMON)</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>DDR356294A</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>DEE DEE SHAMPOO (RF) - STRAWBERRY BTL/250ML (POKEMON)</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>DDR356491A</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>DEE DEE SHAMPOO - APPLE BTL/125ML (POKEMON)</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>DDR356492A</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>DEE DEE SHAMPOO - GRAPE BTL/125ML (POKEMON)</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>DDR356493A</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>DEE DEE SHAMPOO - ORANGE BTL/125ML (POKEMON)</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>DDR356494A</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>DEE DEE SHAMPOO - STRAWBERRY BTL/125ML (POKEMON)</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>DDR356991A</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>DEE DEE SHAMPOO APPLE - POUCH / 200ML (POKEMON)</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>DDR356994A</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>DEE DEE SHAMPOO STRAWBERRY - POUCH / 200ML (POKEMON)</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>DDR356994A-Z01</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>DEE DEE SHAMPOO STRAWBERRY - POUCH/200 ML BELI1 GRATIS1</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>DDS356072</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>DEEDEE SHAMPOO  GRAPE /5ML</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>DDS356073</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>DEEDEE SHAMPOO  ORANGE /5ML</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>DDS992283A</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>DEEDEE SHAMPOO GREEN TEA PUMP/200ML</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>DFW662092</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>DEEDEE FACIAL WASH GRAPE /100ML</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>DFW662093</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>DEEDEE FACIAL WASH ORANGE /100ML</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>DFW662094</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>DEEDEE FACIAL WASH STRAWBERRY /100ML</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>DFW662193</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>DEEDEE FACIAL WASH ORANGE /50GR</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>DFW662902</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>DEEDEE FACIAL WASH GRAPE /50GR</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>DFW662904</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>DEEDEE FACIAL WASH STRAWBERRY /50GR</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>DPK442282C</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>DEDEE TOOTH PASTE-POKEMON GRAPE TM/50GR</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>DPK442283C</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>DEDEE TOOTH PASTE-POKEMON ORANGE TM/50GR</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>DPK442284C</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>DEDEE TOOTH PASTE-POKEMON STRAWBERRY TM/50GR</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>DPS442267</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>DEEDEE T.BRUSH +T.PASTE 50GR MIX TM</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>DPT464267</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>DEEDEE TRAVEL PACK MIX</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>DSG442492</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>DEEDEE TOOTH BRUSH MIX /TRAY</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>DSG442590</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>DEEDEE TOOTH BRUSH  BOX KECIL</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>DTP464191-Z01</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>DEEDEE TALCUM POWDER APPLE /45GR</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>DTP464193-Z01</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>DEEDEE TALCUM POWDER ORANGE /45GR</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>DTP464194-Z01</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>DEEDEE TALCUM POWDER STRAWBERRY /45GR</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>DTP464291-Z01</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>DEE DEE TALCUM POWDER - APPLE BTL/ 150GR + FREE FOAM STIKER CAR</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>DTP464293-Z01</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>DEE DEE TALCUM POWDER - ORANGE BTL/ 150GR + FREE FOAM STIKER CAR</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>DTP464294-Z01</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>DEE DEE TALCUM POWDER - STRAWBERRY BTL/ 150GR + FREE FOAM STIKER CAR</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>GLA178280</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>YURI GLASS CLEANER FOAMING FRESH BLUE SPRAY/500ML</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>GLA178282</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>YURI GLASS CLEANER FOAMING LEMON SPRAY/500ML</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>GLA178283</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>YURI GLASS CLEANER FOAMING FRESH LILAC SPRAY/500ML</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>GLA178592</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>YURI GLASS CLEANER FOAMING LEMON FRESH /3,7LT</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>GLA178593</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>YURI GLASS CLEANER FOAMING FRESH LILAC /3,7LT</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>GLA178990</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>YURI GLASS CLEANER FOAMING FRESH BLUE /410ML</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>GLA178992</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>YURI GLASS CLEANER FOAMING LEMON FRESH /410ML</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>GLA178993</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>YURI GLASS CLEANER FOAMING LILAC  /410ML</t>
+        </is>
+      </c>
+      <c r="C86" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>HSA981283A</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>YURI HAND SOAP FOAMING GREEN TEA /410ML</t>
+        </is>
+      </c>
+      <c r="C87" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>HSA981283A-Z02</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>YURI HAND SOAP FOAMING GREEN TEA /410ML FREE HAND GEL 50ML</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>HSA981993A</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>YURI HAND SOAP FOAMING GREEN TEA /375ML</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>HSA981995A</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>YURI HAND SOAP FOAMING LAVANDER /375ML</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>HSP222381</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>YURI HAND SOAP APPLE PUMP /410ML</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>HSP222383</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>YURI HAND SOAP GRAPES PUMP /410ML</t>
+        </is>
+      </c>
+      <c r="C92" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>HSP222384</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>YURI HAND SOAP LEMON PUMP /410ML</t>
+        </is>
+      </c>
+      <c r="C93" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>HSP222385</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>YURI HAND SOAP ORANGE PUMP /410ML</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>HSP222386</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>YURI HAND SOAP STRAWBERRY PUMP /410ML</t>
+        </is>
+      </c>
+      <c r="C95" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>HSP223301A</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>YURI HAND SOAP LAVENDER FOAMING PUMP/410ML</t>
+        </is>
+      </c>
+      <c r="C96" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>HSR222591</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>YURI HAND SOAP APPLE  /3,7LT</t>
+        </is>
+      </c>
+      <c r="C97" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>HSR222593</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>YURI HAND SOAP GRAPE  /3,7LT</t>
+        </is>
+      </c>
+      <c r="C98" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>HSR222594</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>YURI HAND SOAP LEMON  /3,7LT</t>
+        </is>
+      </c>
+      <c r="C99" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>HSR222595</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>YURI HAND SOAP ORANGE  /3,7LT</t>
+        </is>
+      </c>
+      <c r="C100" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>HSR222596</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>YURI HAND SOAP STRAWBERRY  /3,7LT</t>
+        </is>
+      </c>
+      <c r="C101" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>HSR222991</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>YURI HAND SOAP APPLE  /375ML</t>
+        </is>
+      </c>
+      <c r="C102" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>HSR222993</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>YURI HAND SOAP GRAPE  /375ML</t>
+        </is>
+      </c>
+      <c r="C103" t="n">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>HSR222994</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>YURI HAND SOAP LEMON  /375ML</t>
+        </is>
+      </c>
+      <c r="C104" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>HSR222995</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>YURI HAND SOAP ORANGE  /375ML</t>
+        </is>
+      </c>
+      <c r="C105" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>HSR222996</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>YURI HAND SOAP STRAW  /375ML</t>
+        </is>
+      </c>
+      <c r="C106" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>HSR222996-Z01</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>YURI HAND SOAP STRAW /375ML</t>
+        </is>
+      </c>
+      <c r="C107" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>LIB257381</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>LIGENT BABY PUMP /450ML FREE GIFT</t>
+        </is>
+      </c>
+      <c r="C108" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>LIB257991</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>LIGENT BABY POUCH /410ML</t>
+        </is>
+      </c>
+      <c r="C109" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>LIG252481-Z01</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>LIGENT LIME PUMP /1L + CUP COVER</t>
+        </is>
+      </c>
+      <c r="C110" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>LIG252482-Z01</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>LIGENT LEMON PUMP /1L + CUP COVER</t>
+        </is>
+      </c>
+      <c r="C111" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>LIG252495-Z01</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>LIGENT GRAPEFRUIT  /1L + CUP COVER</t>
+        </is>
+      </c>
+      <c r="C112" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>LIG252591</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>LIGENT LIME  /3,7LT</t>
+        </is>
+      </c>
+      <c r="C113" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>LIG252592</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>LIGENT LEMON  /3,7LT</t>
+        </is>
+      </c>
+      <c r="C114" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>LIG252921C-Z01</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>LIGENT BIO  LIME &amp; BERGAMOT /600ML BELI 1 GRATIS 1</t>
+        </is>
+      </c>
+      <c r="C115" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>LIG252922C-Z01</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>LIGENT BIO  LEMON &amp; BERGAMOT /600ML BELI 1 GRATIS 1</t>
+        </is>
+      </c>
+      <c r="C116" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>LIG252925C-Z01</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>LIGENT BIO  GRAPEFRUIT &amp; BERGAMOT /600ML BELI 1 GRATIS 1</t>
+        </is>
+      </c>
+      <c r="C117" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>LYS277280</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>LYSORIN   /630ML</t>
+        </is>
+      </c>
+      <c r="C118" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>LYS277390</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>LYSORIN   /1L</t>
+        </is>
+      </c>
+      <c r="C119" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>MAT211392</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>YURIMATIC COLOUR  /1KG</t>
+        </is>
+      </c>
+      <c r="C120" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>MAT211453A</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>YUTIMATIC 1.8KG LOW SUD + TRIL SPRAY 500ML</t>
+        </is>
+      </c>
+      <c r="C121" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>MAT211941</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>YURIMATIC TOUGH STAIN  /1.8KG</t>
+        </is>
+      </c>
+      <c r="C122" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>MAT211991</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>YURIMATIC TOUGH STAIN  /630GR</t>
+        </is>
+      </c>
+      <c r="C123" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>MAT211992</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>YURIMATIC COLOUR  /630GR</t>
+        </is>
+      </c>
+      <c r="C124" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>MAT211993</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>YURIMATIC LOW SUDS  /630GR</t>
+        </is>
+      </c>
+      <c r="C125" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>NaN</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>NaN</t>
+        </is>
+      </c>
+      <c r="C126" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>POR332090</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>YURI PRSTX BIRU 1000(+PORS160)</t>
+        </is>
+      </c>
+      <c r="C127" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>POR332270</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>PORSTEX KLOSET  /500ML</t>
+        </is>
+      </c>
+      <c r="C128" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>POR332290</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>PORSTEX BIRU  /500ML</t>
+        </is>
+      </c>
+      <c r="C129" t="n">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>POR332390</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>PORSTEX BIRU  /1L</t>
+        </is>
+      </c>
+      <c r="C130" t="n">
+        <v>718</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>POR332490</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>PORSTEX BIRU  /2L</t>
+        </is>
+      </c>
+      <c r="C131" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>POR332590</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>PORSTEX BIRU  /3,7LT</t>
+        </is>
+      </c>
+      <c r="C132" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>POU332280</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>PORSTEX UNGU(WB)  /500ML</t>
+        </is>
+      </c>
+      <c r="C133" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>POU332380</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>PORSTEX UNGU(WB)  /1L</t>
+        </is>
+      </c>
+      <c r="C134" t="n">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>POU332480</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>PORSTEX UNGU(WB)  /2L</t>
+        </is>
+      </c>
+      <c r="C135" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>POU332580</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>PORSTEX UNGU(WB)  /3,7LT</t>
+        </is>
+      </c>
+      <c r="C136" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>PSR563290</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>YURI PORSTEX REGULER OCEAN BLUE / 160ML EXTRA 40ML</t>
+        </is>
+      </c>
+      <c r="C137" t="n">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>PSR563380</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>PORSTEX REGULAR  LILAC FRESH /700ML</t>
+        </is>
+      </c>
+      <c r="C138" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>PSR563390</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>PORSTEX REGULAR OCEAN BLUE /700ML</t>
+        </is>
+      </c>
+      <c r="C139" t="n">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>SOL420990</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>YURISOL   /630ML</t>
+        </is>
+      </c>
+      <c r="C140" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>TAF365280</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>TAF KITCHEN CLEANER SPRAY /500ML</t>
+        </is>
+      </c>
+      <c r="C141" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>TAF365391</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>TAF LEMON &amp; LIME FLIPTOP /500ML</t>
+        </is>
+      </c>
+      <c r="C142" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>TAF365480</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>TAF KITCHEN CLEANER 500ML SPRAY +RF /500ML</t>
+        </is>
+      </c>
+      <c r="C143" t="n">
+        <v>-171</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>TAF365490</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>TAF KITCHEN CLEANER  /375ML</t>
+        </is>
+      </c>
+      <c r="C144" t="n">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C174"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Kode SKU JIM</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Nama SKU JIM</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Avg Qty Outsell Karton</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>AGA080391</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>AGANOL LAVENDER  /1L</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>AGA080591</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>AGANOL LAVENDER  /3,7LT</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>AGA080991</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>AGANOL LAVENDER  /630ML</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>AGA080991-Z01</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>AGANOL LAVENDER /600ML + BUY 1 GET 1</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>AGA101391A</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>AGANOL FLORAL  /1L</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>AGA101392</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>AGANOL LEMON FRESH  /1L</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>AGA101393</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>AGANOL MORNING FRESH W/ LEMONGRASS  /1L</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>AGA101491A</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>AGANOL FLORAL  /2L</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>AGA101492</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>AGANOL LEMON FRESH  /2L</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>AGA101493</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>AGANOL MORNING FRESH W/ LEMONGRASS  /2L</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>AGA101591</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>AGANOL FLORAL  /3,7LT</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>AGA101593</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>AGANOL MORNING FRESH W/ LEMONGRASS  /3,7LT</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>AGA101991B</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>AGANOL FLORAL  /630ML</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>AGA101992</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>AGANOL LEMON  /630ML</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>AGA101993</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>AGANOL MORNING FRESH W/ LEMONGRASS  /630ML</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>BBS106390</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>BABY SOFT   /1L</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>BBS106590</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>BABY SOFT   /3,7LT</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>BCL100280</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>YURI BATHROOM CLEANER   /500ML</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>BCL100390</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>YURI BATHROOM CLEANER   /375ML</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>BIO112290</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>BIOSOFT   /375ML</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>BIO112590</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>BIOSOFT   /3,7LT</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>BIO113921</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>BIOSOFT HIJAB DETERGENT+SOFTENER OCEAN FRESH /630ML</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>BIO114921</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>BIOSOFT HIJAB PEWANGI+SOFTENER OCEAN FRESH /630ML</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>BLE123390</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>YURI BLEACH MORNING FRESH  /1L</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>BLE123392</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>YURI BLEACH LEMON  /1L</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>BLE123590</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>YURI BLEACH MORNING FRESH  /3,7LT</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>BLE123592</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>YURI BLEACH LEMON  /3,7LT</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>DBD750291</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>BABYDEE BODYWASH &amp; SHAMPOO MILK /200ML</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>DBD750292</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>BABYDEE BODYWASH &amp; SHAMPOO HONEY /200ML</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>DBD750931</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>BABY DEE BODYWASH &amp; SHAMPOO NATURAL MILK &amp; LAVENDER EXTRACT FOAMING 600ML</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>DBD750932</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>BABY DEE BODYWASH &amp; SHAMPOO NATURAL HONEY&amp;CHAMOMILE EXTRACT FOAMING 600ML</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>DBD761261</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>BABYDEE TRAVEL PACK MILK</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>DBD761262</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>BABYDEE TRAVEL PACK HONEY</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>DBD761291</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>BABYDEE TALCUM MILK /200GR</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>DBD761292</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>BABYDEE TALCUM HONEY /200GR</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>DBD789091</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>BABYDEE DIAPER CREAM MILK /50GR</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>DBD789092</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>BABYDEE DIAPER CREAM HONEY /50GR</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>DBD789192</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>BABYDEE DIAPER CREAM HONEY /100GR</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>DBD794091</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>BABYDEE BABY LOTION MILK /50ML</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>DBD794092</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>BABYDEE BABY LOTION HONEY /50ML</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>DBD794191</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>BABYDEE BABY LOTION MILK /100ML</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>DBW640291</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>DEEDEE BODYWASH APPLE /225ML</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>DBW640292</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>DEEDEE BODYWASH GRAPE /225ML</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>DBW640293</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>DEEDEE BODYWASH ORANGE /225ML</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>DBW640294</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>DEEDEE BODYWASH STRAWBERRY /225ML</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>DBW640991</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>DEEDEE BODYWASH APPLE /200ML</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>DBW640992</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>DEEDEE BODYWASH GRAPE /200ML</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>DBW640993</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>DEEDEE BODYWASH ORANGE /200ML</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>DBW640994</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>DEEDEE BODYWASH STRAWBERRY /200ML</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>DDM497074</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>DEEDEE LOT.PENOLAK NYAMUK STRAW. /5ML</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>DDM497193</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>DEEDEE LOT. PENOLAK NYAMUK ORANGE /50GR</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>DDM497195</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>DEEDEE LOT. PENOLAK NYAMUK GUAVA /50GR</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>DDP356281A</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>DEE DEE SHAMPOO (P) - APPLE BTL/250ML (POKEMON)</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>DDP356282A</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>DEE DEE SHAMPOO (P) - GRAPE BTL/250ML (POKEMON)</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>DDP356283A</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>DEE DEE SHAMPOO (P) - ORANGE BTL/250ML (POKEMON)</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>DDP356284A</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>DEE DEE SHAMPOO (P) - STRAWBERRY BTL/250ML (POKEMON)</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>DDR356191A</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>DEEDEE SHAMPOO APPLE /45ML</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>DDR356192A</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>DEEDEE SHAMPOO GRAPE /45ML</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>DDR356193A</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>DEEDEE SHAMPOO ORANGE /45ML</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>DDR356194A</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>DEEDEE SHAMPOO STRAWBERRY /45ML</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>DDR356291A</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>DEE DEE SHAMPOO (RF) - APPLE BTL/250ML (POKEMON)</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>DDR356292A</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>DEE DEE SHAMPOO (RF) - GRAPE BTL/250ML (POKEMON)</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>DDR356293A</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>DEE DEE SHAMPOO (RF) - ORANGE BTL/250ML (POKEMON)</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>DDR356294A</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>DEE DEE SHAMPOO (RF) - STRAWBERRY BTL/250ML (POKEMON)</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>DDR356491A</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>DEE DEE SHAMPOO - APPLE BTL/125ML (POKEMON)</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>DDR356492A</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>DEE DEE SHAMPOO - GRAPE BTL/125ML (POKEMON)</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>DDR356493A</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>DEE DEE SHAMPOO - ORANGE BTL/125ML (POKEMON)</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>DDR356494A</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>DEE DEE SHAMPOO - STRAWBERRY BTL/125ML (POKEMON)</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>DDR356991A</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>DEE DEE SHAMPOO APPLE - POUCH / 200ML (POKEMON)</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>DDR356994A</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>DEE DEE SHAMPOO STRAWBERRY - POUCH / 200ML (POKEMON)</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>DDR356994A-Z01</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>DEE DEE SHAMPOO STRAWBERRY - POUCH/200 ML BELI1 GRATIS1</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>DDS356072</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>DEEDEE SHAMPOO  GRAPE /5ML</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>DDS356073</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>DEEDEE SHAMPOO  ORANGE /5ML</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>DDS992283A</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>DEEDEE SHAMPOO GREEN TEA PUMP/200ML</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>DDS992284A</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>DEEDEE SHAMPOO ROSE PUMP/200ML</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>DFW662092</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>DEEDEE FACIAL WASH GRAPE /100ML</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>DFW662093</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>DEEDEE FACIAL WASH ORANGE /100ML</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>DFW662094</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>DEEDEE FACIAL WASH STRAWBERRY /100ML</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>DFW662193</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>DEEDEE FACIAL WASH ORANGE /50GR</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>DFW662902</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>DEEDEE FACIAL WASH GRAPE /50GR</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>DFW662904</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>DEEDEE FACIAL WASH STRAWBERRY /50GR</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>DPK442282C</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>DEDEE TOOTH PASTE-POKEMON GRAPE TM/50GR</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>DPK442283C</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>DEDEE TOOTH PASTE-POKEMON ORANGE TM/50GR</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>DPK442284C</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>DEDEE TOOTH PASTE-POKEMON STRAWBERRY TM/50GR</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>DPS442267</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>DEEDEE T.BRUSH +T.PASTE 50GR MIX TM</t>
+        </is>
+      </c>
+      <c r="C86" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>DPT464267</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>DEEDEE TRAVEL PACK MIX</t>
+        </is>
+      </c>
+      <c r="C87" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>DSG442482</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>DEEDEE TOOTH BRUSH MIX /HANGER</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>DSG442492</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>DEEDEE TOOTH BRUSH MIX /TRAY</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>DSG442590</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>DEEDEE TOOTH BRUSH  BOX KECIL</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>DTP464191-Z01</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>DEEDEE TALCUM POWDER APPLE /45GR</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>DTP464193-Z01</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>DEEDEE TALCUM POWDER ORANGE /45GR</t>
+        </is>
+      </c>
+      <c r="C92" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>DTP464194-Z01</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>DEEDEE TALCUM POWDER STRAWBERRY /45GR</t>
+        </is>
+      </c>
+      <c r="C93" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>DTP464291-Z01</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>DEE DEE TALCUM POWDER - APPLE BTL/ 150GR + FREE FOAM STIKER CAR</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>DTP464293-Z01</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>DEE DEE TALCUM POWDER - ORANGE BTL/ 150GR + FREE FOAM STIKER CAR</t>
+        </is>
+      </c>
+      <c r="C95" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>DTP464294-Z01</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>DEE DEE TALCUM POWDER - STRAWBERRY BTL/ 150GR + FREE FOAM STIKER CAR</t>
+        </is>
+      </c>
+      <c r="C96" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>GLA178280</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>YURI GLASS CLEANER FOAMING FRESH BLUE SPRAY/500ML</t>
+        </is>
+      </c>
+      <c r="C97" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>GLA178282</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>YURI GLASS CLEANER FOAMING LEMON SPRAY/500ML</t>
+        </is>
+      </c>
+      <c r="C98" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>GLA178283</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>YURI GLASS CLEANER FOAMING FRESH LILAC SPRAY/500ML</t>
+        </is>
+      </c>
+      <c r="C99" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>GLA178590</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>YURI GLASS CLEANER FOAMING FRESH BLUE /3,7LT</t>
+        </is>
+      </c>
+      <c r="C100" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>GLA178592</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>YURI GLASS CLEANER FOAMING LEMON FRESH /3,7LT</t>
+        </is>
+      </c>
+      <c r="C101" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>GLA178593</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>YURI GLASS CLEANER FOAMING FRESH LILAC /3,7LT</t>
+        </is>
+      </c>
+      <c r="C102" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>GLA178990</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>YURI GLASS CLEANER FOAMING FRESH BLUE /410ML</t>
+        </is>
+      </c>
+      <c r="C103" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>GLA178992</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>YURI GLASS CLEANER FOAMING LEMON FRESH /410ML</t>
+        </is>
+      </c>
+      <c r="C104" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>GLA178993</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>YURI GLASS CLEANER FOAMING LILAC  /410ML</t>
+        </is>
+      </c>
+      <c r="C105" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>HSA981283A</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>YURI HAND SOAP FOAMING GREEN TEA /410ML</t>
+        </is>
+      </c>
+      <c r="C106" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>HSA981283A-Z02</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>YURI HAND SOAP FOAMING GREEN TEA /410ML FREE HAND GEL 50ML</t>
+        </is>
+      </c>
+      <c r="C107" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>HSA981993A</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>YURI HAND SOAP FOAMING GREEN TEA /375ML</t>
+        </is>
+      </c>
+      <c r="C108" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>HSA981994A</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>YURI HAND SOAP FOAMING ROSE /375ML</t>
+        </is>
+      </c>
+      <c r="C109" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>HSA981995A</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>YURI HAND SOAP FOAMING LAVANDER /375ML</t>
+        </is>
+      </c>
+      <c r="C110" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>HSP222381</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>YURI HAND SOAP APPLE PUMP /410ML</t>
+        </is>
+      </c>
+      <c r="C111" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>HSP222383</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>YURI HAND SOAP GRAPES PUMP /410ML</t>
+        </is>
+      </c>
+      <c r="C112" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>HSP222384</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>YURI HAND SOAP LEMON PUMP /410ML</t>
+        </is>
+      </c>
+      <c r="C113" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>HSP222385</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>YURI HAND SOAP ORANGE PUMP /410ML</t>
+        </is>
+      </c>
+      <c r="C114" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>HSP222386</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>YURI HAND SOAP STRAWBERRY PUMP /410ML</t>
+        </is>
+      </c>
+      <c r="C115" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>HSP222791</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>YURI HAND SOAP APPLE PUMP /410ML FREE HAND SOAP /375ML</t>
+        </is>
+      </c>
+      <c r="C116" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>HSP222796</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>YURI HAND SOAP STRAWBERRY PUMP /410ML FREE HAND SOAP /375ML</t>
+        </is>
+      </c>
+      <c r="C117" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>HSP223301A</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>YURI HAND SOAP LAVENDER FOAMING PUMP/410ML</t>
+        </is>
+      </c>
+      <c r="C118" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>HSR222591</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>YURI HAND SOAP APPLE  /3,7LT</t>
+        </is>
+      </c>
+      <c r="C119" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>HSR222593</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>YURI HAND SOAP GRAPE  /3,7LT</t>
+        </is>
+      </c>
+      <c r="C120" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>HSR222594</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>YURI HAND SOAP LEMON  /3,7LT</t>
+        </is>
+      </c>
+      <c r="C121" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>HSR222595</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>YURI HAND SOAP ORANGE  /3,7LT</t>
+        </is>
+      </c>
+      <c r="C122" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>HSR222596</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>YURI HAND SOAP STRAWBERRY  /3,7LT</t>
+        </is>
+      </c>
+      <c r="C123" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>HSR222991</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>YURI HAND SOAP APPLE  /375ML</t>
+        </is>
+      </c>
+      <c r="C124" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>HSR222991-Z01</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>YURI HAND SOAP APPLE /375ML</t>
+        </is>
+      </c>
+      <c r="C125" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>HSR222993</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>YURI HAND SOAP GRAPE  /375ML</t>
+        </is>
+      </c>
+      <c r="C126" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>HSR222994</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>YURI HAND SOAP LEMON  /375ML</t>
+        </is>
+      </c>
+      <c r="C127" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>HSR222995</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>YURI HAND SOAP ORANGE  /375ML</t>
+        </is>
+      </c>
+      <c r="C128" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>HSR222995-Z01</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>YURI HAND SOAP ORANGE /375ML</t>
+        </is>
+      </c>
+      <c r="C129" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>HSR222996</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>YURI HAND SOAP STRAW  /375ML</t>
+        </is>
+      </c>
+      <c r="C130" t="n">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>HSR222996-Z01</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>YURI HAND SOAP STRAW /375ML</t>
+        </is>
+      </c>
+      <c r="C131" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>LIB257381</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>LIGENT BABY PUMP /450ML FREE GIFT</t>
+        </is>
+      </c>
+      <c r="C132" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>LIB257991</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>LIGENT BABY POUCH /410ML</t>
+        </is>
+      </c>
+      <c r="C133" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>LIG252481-Z01</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>LIGENT LIME PUMP /1L + CUP COVER</t>
+        </is>
+      </c>
+      <c r="C134" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>LIG252482-Z01</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>LIGENT LEMON PUMP /1L + CUP COVER</t>
+        </is>
+      </c>
+      <c r="C135" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>LIG252495-Z01</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>LIGENT GRAPEFRUIT  /1L + CUP COVER</t>
+        </is>
+      </c>
+      <c r="C136" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>LIG252591</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>LIGENT LIME  /3,7LT</t>
+        </is>
+      </c>
+      <c r="C137" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>LIG252592</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>LIGENT LEMON  /3,7LT</t>
+        </is>
+      </c>
+      <c r="C138" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>LIG252921C-Z01</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>LIGENT BIO  LIME &amp; BERGAMOT /600ML BELI 1 GRATIS 1</t>
+        </is>
+      </c>
+      <c r="C139" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>LIG252922C-Z01</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>LIGENT BIO  LEMON &amp; BERGAMOT /600ML BELI 1 GRATIS 1</t>
+        </is>
+      </c>
+      <c r="C140" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>LIG252925C-Z01</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>LIGENT BIO  GRAPEFRUIT &amp; BERGAMOT /600ML BELI 1 GRATIS 1</t>
+        </is>
+      </c>
+      <c r="C141" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>LYS277280</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>LYSORIN   /630ML</t>
+        </is>
+      </c>
+      <c r="C142" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>LYS277390</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>LYSORIN   /1L</t>
+        </is>
+      </c>
+      <c r="C143" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>LYS277590</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>LYSORIN   /3,7LT</t>
+        </is>
+      </c>
+      <c r="C144" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>MAT211392</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>YURIMATIC COLOUR  /1KG</t>
+        </is>
+      </c>
+      <c r="C145" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>MAT211453A</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>YUTIMATIC 1.8KG LOW SUD + TRIL SPRAY 500ML</t>
+        </is>
+      </c>
+      <c r="C146" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>MAT211941</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>YURIMATIC TOUGH STAIN  /1.8KG</t>
+        </is>
+      </c>
+      <c r="C147" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>MAT211991</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>YURIMATIC TOUGH STAIN  /630GR</t>
+        </is>
+      </c>
+      <c r="C148" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>MAT211992</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>YURIMATIC COLOUR  /630GR</t>
+        </is>
+      </c>
+      <c r="C149" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>MAT211993</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>YURIMATIC LOW SUDS  /630GR</t>
+        </is>
+      </c>
+      <c r="C150" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>NaN</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>NaN</t>
+        </is>
+      </c>
+      <c r="C151" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>POR332090</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>YURI PRSTX BIRU 1000(+PORS160)</t>
+        </is>
+      </c>
+      <c r="C152" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>POR332270</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>PORSTEX KLOSET  /500ML</t>
+        </is>
+      </c>
+      <c r="C153" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>POR332290</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>PORSTEX BIRU  /500ML</t>
+        </is>
+      </c>
+      <c r="C154" t="n">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>POR332390</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>PORSTEX BIRU  /1L</t>
+        </is>
+      </c>
+      <c r="C155" t="n">
+        <v>703</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>POR332490</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>PORSTEX BIRU  /2L</t>
+        </is>
+      </c>
+      <c r="C156" t="n">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>POR332590</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>PORSTEX BIRU  /3,7LT</t>
+        </is>
+      </c>
+      <c r="C157" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>POU332280</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>PORSTEX UNGU(WB)  /500ML</t>
+        </is>
+      </c>
+      <c r="C158" t="n">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>POU332380</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>PORSTEX UNGU(WB)  /1L</t>
+        </is>
+      </c>
+      <c r="C159" t="n">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>POU332480</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>PORSTEX UNGU(WB)  /2L</t>
+        </is>
+      </c>
+      <c r="C160" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>POU332580</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>PORSTEX UNGU(WB)  /3,7LT</t>
+        </is>
+      </c>
+      <c r="C161" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>PSR563290</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>YURI PORSTEX REGULER OCEAN BLUE / 160ML EXTRA 40ML</t>
+        </is>
+      </c>
+      <c r="C162" t="n">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>PSR563380</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>PORSTEX REGULAR  LILAC FRESH /700ML</t>
+        </is>
+      </c>
+      <c r="C163" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>PSR563390</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>PORSTEX REGULAR OCEAN BLUE /700ML</t>
+        </is>
+      </c>
+      <c r="C164" t="n">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>SOL420390</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>YURISOL   /1L</t>
+        </is>
+      </c>
+      <c r="C165" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>SOL420990</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>YURISOL   /630ML</t>
+        </is>
+      </c>
+      <c r="C166" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>TAF365280</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>TAF KITCHEN CLEANER SPRAY /500ML</t>
+        </is>
+      </c>
+      <c r="C167" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>TAF365391</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>TAF LEMON &amp; LIME FLIPTOP /500ML</t>
+        </is>
+      </c>
+      <c r="C168" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>TAF365480</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>TAF KITCHEN CLEANER 500ML SPRAY +RF /500ML</t>
+        </is>
+      </c>
+      <c r="C169" t="n">
+        <v>-31</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>TAF365490</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>TAF KITCHEN CLEANER  /375ML</t>
+        </is>
+      </c>
+      <c r="C170" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>TRI431990</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>TRIL ROMANTIC BLUE REFILL /410ML</t>
+        </is>
+      </c>
+      <c r="C171" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>TRI431992</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>TRIL FLORAL REFILL /410ML</t>
+        </is>
+      </c>
+      <c r="C172" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>TRI431993</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>TRIL LAVENDER REFILL /410ML</t>
+        </is>
+      </c>
+      <c r="C173" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>YDS370280-Z03</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>YURI DISINFECTANT SPRAY /500ML +50ML</t>
+        </is>
+      </c>
+      <c r="C174" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>